<commit_message>
Organize draft reports and improve script outputs
</commit_message>
<xml_diff>
--- a/trade-elasticities-cointegration/outputs/13_outputs_index/final_outputs_index.xlsx
+++ b/trade-elasticities-cointegration/outputs/13_outputs_index/final_outputs_index.xlsx
@@ -463,7 +463,7 @@
         <v>27.6</v>
       </c>
       <c r="J2" s="2">
-        <v>46192.07709149623</v>
+        <v>46199.12516088157</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
         <v>22.6</v>
       </c>
       <c r="J3" s="2">
-        <v>46192.07709249128</v>
+        <v>46199.12516458145</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         <v>74.8</v>
       </c>
       <c r="J4" s="2">
-        <v>46192.07710595173</v>
+        <v>46199.12518203027</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         <v>81.2</v>
       </c>
       <c r="J5" s="2">
-        <v>46192.07711189142</v>
+        <v>46199.12518636062</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         <v>80.09999999999999</v>
       </c>
       <c r="J6" s="2">
-        <v>46192.07754922443</v>
+        <v>46199.12551652463</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>212.9</v>
       </c>
       <c r="J7" s="2">
-        <v>46192.07728301523</v>
+        <v>46199.12532896885</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
         <v>224.2</v>
       </c>
       <c r="J8" s="2">
-        <v>46192.07730258211</v>
+        <v>46199.12534871408</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -820,7 +820,7 @@
         <v>426.7</v>
       </c>
       <c r="J9" s="2">
-        <v>46192.07731982241</v>
+        <v>46199.12536001062</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>284.6</v>
       </c>
       <c r="J10" s="2">
-        <v>46192.07734197787</v>
+        <v>46199.12537558941</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>61.2</v>
       </c>
       <c r="J11" s="2">
-        <v>46192.07735633835</v>
+        <v>46199.12538315718</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         <v>261.7</v>
       </c>
       <c r="J12" s="2">
-        <v>46192.07767751065</v>
+        <v>46199.12565999219</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         <v>338.3</v>
       </c>
       <c r="J13" s="2">
-        <v>46192.07769750412</v>
+        <v>46199.12567139151</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
         <v>98.5</v>
       </c>
       <c r="J14" s="2">
-        <v>46192.07770781877</v>
+        <v>46199.12567676551</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>174.9</v>
       </c>
       <c r="J15" s="2">
-        <v>46192.07772350252</v>
+        <v>46199.1256842511</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         <v>62.2</v>
       </c>
       <c r="J16" s="2">
-        <v>46192.07773420601</v>
+        <v>46199.12569023964</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         <v>13.1</v>
       </c>
       <c r="J17" s="2">
-        <v>46192.07738451715</v>
+        <v>46199.12540908418</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1279,7 +1279,7 @@
         <v>19.3</v>
       </c>
       <c r="J18" s="2">
-        <v>46192.07755038553</v>
+        <v>46199.12553252997</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1330,7 +1330,7 @@
         <v>26.9</v>
       </c>
       <c r="J19" s="2">
-        <v>46192.07764681101</v>
+        <v>46199.12563261211</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         <v>10.3</v>
       </c>
       <c r="J20" s="2">
-        <v>46192.07766089936</v>
+        <v>46199.12564948583</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1432,7 +1432,7 @@
         <v>0.7</v>
       </c>
       <c r="J21" s="2">
-        <v>46192.07764469484</v>
+        <v>46199.12560009828</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
         <v>1.4</v>
       </c>
       <c r="J22" s="2">
-        <v>46192.07764552119</v>
+        <v>46199.12560151864</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1534,7 +1534,7 @@
         <v>9.300000000000001</v>
       </c>
       <c r="J23" s="2">
-        <v>46190.63081018519</v>
+        <v>46192.07774213197</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v>9.1</v>
       </c>
       <c r="J24" s="2">
-        <v>46190.63081018519</v>
+        <v>46192.07774805387</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -1633,10 +1633,10 @@
         <v>1</v>
       </c>
       <c r="I25">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="J25" s="2">
-        <v>46190.63081018519</v>
+        <v>46192.08180824898</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -1684,10 +1684,10 @@
         <v>1</v>
       </c>
       <c r="I26">
-        <v>2488.3</v>
+        <v>2224.7</v>
       </c>
       <c r="J26" s="2">
-        <v>46190.63081018519</v>
+        <v>46198.91592566972</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -1780,10 +1780,10 @@
         <v>1</v>
       </c>
       <c r="I28">
-        <v>142</v>
+        <v>149.9</v>
       </c>
       <c r="J28" s="2">
-        <v>46192.07463526068</v>
+        <v>46199.11970547312</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Organize econometrics project deliverables
</commit_message>
<xml_diff>
--- a/trade-elasticities-cointegration/outputs/13_outputs_index/final_outputs_index.xlsx
+++ b/trade-elasticities-cointegration/outputs/13_outputs_index/final_outputs_index.xlsx
@@ -433,7 +433,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -453,7 +453,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/trade_elasticities_panel_2004_2025.dta</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_2004_2025.dta</t>
         </is>
       </c>
       <c r="H2" t="b">
@@ -463,7 +463,7 @@
         <v>27.6</v>
       </c>
       <c r="J2" s="2">
-        <v>46199.12516088157</v>
+        <v>46210.58626294244</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/trade_elasticities_panel_2004_2025.csv</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_2004_2025.csv</t>
         </is>
       </c>
       <c r="H3" t="b">
@@ -514,7 +514,7 @@
         <v>22.6</v>
       </c>
       <c r="J3" s="2">
-        <v>46199.12516458145</v>
+        <v>46210.58626618114</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/trade_elasticities_panel_transformed_2004_2025.dta</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_transformed_2004_2025.dta</t>
         </is>
       </c>
       <c r="H4" t="b">
@@ -565,7 +565,7 @@
         <v>74.8</v>
       </c>
       <c r="J4" s="2">
-        <v>46199.12518203027</v>
+        <v>46210.58627464592</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -586,7 +586,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/final_data_panel</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/trade_elasticities_panel_transformed_2004_2025.csv</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/final_data_panel/trade_elasticities_panel_transformed_2004_2025.csv</t>
         </is>
       </c>
       <c r="H5" t="b">
@@ -616,7 +616,7 @@
         <v>81.2</v>
       </c>
       <c r="J5" s="2">
-        <v>46199.12518636062</v>
+        <v>46210.58627715813</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/trade_elasticities_panel_modeling_2004_2025.dta</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_modeling_2004_2025.dta</t>
         </is>
       </c>
       <c r="H6" t="b">
@@ -667,7 +667,7 @@
         <v>80.09999999999999</v>
       </c>
       <c r="J6" s="2">
-        <v>46199.12551652463</v>
+        <v>46210.58646104788</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>212.9</v>
       </c>
       <c r="J7" s="2">
-        <v>46199.12532896885</v>
+        <v>46210.58631514463</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
         <v>224.2</v>
       </c>
       <c r="J8" s="2">
-        <v>46199.12534871408</v>
+        <v>46210.58632507216</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -820,7 +820,7 @@
         <v>426.7</v>
       </c>
       <c r="J9" s="2">
-        <v>46199.12536001062</v>
+        <v>46210.58633319821</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>284.6</v>
       </c>
       <c r="J10" s="2">
-        <v>46199.12537558941</v>
+        <v>46210.58634356819</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>61.2</v>
       </c>
       <c r="J11" s="2">
-        <v>46199.12538315718</v>
+        <v>46210.58634993322</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         <v>261.7</v>
       </c>
       <c r="J12" s="2">
-        <v>46199.12565999219</v>
+        <v>46210.58657387071</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         <v>338.3</v>
       </c>
       <c r="J13" s="2">
-        <v>46199.12567139151</v>
+        <v>46210.58658368576</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
         <v>98.5</v>
       </c>
       <c r="J14" s="2">
-        <v>46199.12567676551</v>
+        <v>46210.58658874137</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>174.9</v>
       </c>
       <c r="J15" s="2">
-        <v>46199.1256842511</v>
+        <v>46210.58659548644</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         <v>62.2</v>
       </c>
       <c r="J16" s="2">
-        <v>46199.12569023964</v>
+        <v>46210.58660012462</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         <v>13.1</v>
       </c>
       <c r="J17" s="2">
-        <v>46199.12540908418</v>
+        <v>46210.5863767195</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1279,7 +1279,7 @@
         <v>19.3</v>
       </c>
       <c r="J18" s="2">
-        <v>46199.12553252997</v>
+        <v>46210.58647334158</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1330,7 +1330,7 @@
         <v>26.9</v>
       </c>
       <c r="J19" s="2">
-        <v>46199.12563261211</v>
+        <v>46210.58655444042</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         <v>10.3</v>
       </c>
       <c r="J20" s="2">
-        <v>46199.12564948583</v>
+        <v>46210.58656659568</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1432,7 +1432,7 @@
         <v>0.7</v>
       </c>
       <c r="J21" s="2">
-        <v>46199.12560009828</v>
+        <v>46210.58652987816</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
         <v>1.4</v>
       </c>
       <c r="J22" s="2">
-        <v>46199.12560151864</v>
+        <v>46210.58653156165</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1531,10 +1531,10 @@
         <v>1</v>
       </c>
       <c r="I23">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="J23" s="2">
-        <v>46192.07774213197</v>
+        <v>46199.12570188512</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v>9.1</v>
       </c>
       <c r="J24" s="2">
-        <v>46192.07774805387</v>
+        <v>46199.12571123514</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -1633,10 +1633,10 @@
         <v>1</v>
       </c>
       <c r="I25">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="J25" s="2">
-        <v>46192.08180824898</v>
+        <v>46199.12571191258</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -1780,10 +1780,10 @@
         <v>1</v>
       </c>
       <c r="I28">
-        <v>149.9</v>
+        <v>150.4</v>
       </c>
       <c r="J28" s="2">
-        <v>46199.11970547312</v>
+        <v>46210.58447072034</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finalize trade elasticity project outputs
</commit_message>
<xml_diff>
--- a/trade-elasticities-cointegration/outputs/13_outputs_index/final_outputs_index.xlsx
+++ b/trade-elasticities-cointegration/outputs/13_outputs_index/final_outputs_index.xlsx
@@ -433,7 +433,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
+          <t>C:/Users/julla/AppData/Local/Temp/RtmpWqAhme/tp2_auxiliary_data</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -453,7 +453,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_2004_2025.dta</t>
+          <t>C:/Users/julla/AppData/Local/Temp/RtmpWqAhme/tp2_auxiliary_data/trade_elasticities_panel_2004_2025.dta</t>
         </is>
       </c>
       <c r="H2" t="b">
@@ -463,7 +463,7 @@
         <v>27.6</v>
       </c>
       <c r="J2" s="2">
-        <v>46210.58626294244</v>
+        <v>46211.00141841756</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
+          <t>C:/Users/julla/AppData/Local/Temp/RtmpWqAhme/tp2_auxiliary_data</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_2004_2025.csv</t>
+          <t>C:/Users/julla/AppData/Local/Temp/RtmpWqAhme/tp2_auxiliary_data/trade_elasticities_panel_2004_2025.csv</t>
         </is>
       </c>
       <c r="H3" t="b">
@@ -514,7 +514,7 @@
         <v>22.6</v>
       </c>
       <c r="J3" s="2">
-        <v>46210.58626618114</v>
+        <v>46211.00142043639</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/final_data_panel</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_transformed_2004_2025.dta</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/final_data_panel/trade_elasticities_panel_transformed_2004_2025.dta</t>
         </is>
       </c>
       <c r="H4" t="b">
@@ -565,7 +565,7 @@
         <v>74.8</v>
       </c>
       <c r="J4" s="2">
-        <v>46210.58627464592</v>
+        <v>46211.00142907421</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         <v>81.2</v>
       </c>
       <c r="J5" s="2">
-        <v>46210.58627715813</v>
+        <v>46211.00143264662</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data</t>
+          <t>C:/Users/julla/AppData/Local/Temp/RtmpWqAhme/tp2_auxiliary_data</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/data/processed/auxiliary_data/trade_elasticities_panel_modeling_2004_2025.dta</t>
+          <t>C:/Users/julla/AppData/Local/Temp/RtmpWqAhme/tp2_auxiliary_data/trade_elasticities_panel_modeling_2004_2025.dta</t>
         </is>
       </c>
       <c r="H6" t="b">
@@ -667,7 +667,7 @@
         <v>80.09999999999999</v>
       </c>
       <c r="J6" s="2">
-        <v>46210.58646104788</v>
+        <v>46211.00158853193</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>212.9</v>
       </c>
       <c r="J7" s="2">
-        <v>46210.58631514463</v>
+        <v>46211.00145020646</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
         <v>224.2</v>
       </c>
       <c r="J8" s="2">
-        <v>46210.58632507216</v>
+        <v>46211.00145876662</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -820,7 +820,7 @@
         <v>426.7</v>
       </c>
       <c r="J9" s="2">
-        <v>46210.58633319821</v>
+        <v>46211.00146703968</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>284.6</v>
       </c>
       <c r="J10" s="2">
-        <v>46210.58634356819</v>
+        <v>46211.0014747742</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>61.2</v>
       </c>
       <c r="J11" s="2">
-        <v>46210.58634993322</v>
+        <v>46211.00147907743</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         <v>261.7</v>
       </c>
       <c r="J12" s="2">
-        <v>46210.58657387071</v>
+        <v>46211.00169085489</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         <v>338.3</v>
       </c>
       <c r="J13" s="2">
-        <v>46210.58658368576</v>
+        <v>46211.00169727838</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
         <v>98.5</v>
       </c>
       <c r="J14" s="2">
-        <v>46210.58658874137</v>
+        <v>46211.00170079814</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>174.9</v>
       </c>
       <c r="J15" s="2">
-        <v>46210.58659548644</v>
+        <v>46211.00170479997</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         <v>62.2</v>
       </c>
       <c r="J16" s="2">
-        <v>46210.58660012462</v>
+        <v>46211.00170791286</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         <v>13.1</v>
       </c>
       <c r="J17" s="2">
-        <v>46210.5863767195</v>
+        <v>46211.00149907183</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1279,7 +1279,7 @@
         <v>19.3</v>
       </c>
       <c r="J18" s="2">
-        <v>46210.58647334158</v>
+        <v>46211.00159772299</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1330,7 +1330,7 @@
         <v>26.9</v>
       </c>
       <c r="J19" s="2">
-        <v>46210.58655444042</v>
+        <v>46211.00167192143</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         <v>10.3</v>
       </c>
       <c r="J20" s="2">
-        <v>46210.58656659568</v>
+        <v>46211.00168481068</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1432,7 +1432,7 @@
         <v>0.7</v>
       </c>
       <c r="J21" s="2">
-        <v>46210.58652987816</v>
+        <v>46211.00164348481</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
         <v>1.4</v>
       </c>
       <c r="J22" s="2">
-        <v>46210.58653156165</v>
+        <v>46211.00164608161</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1534,7 +1534,7 @@
         <v>9.4</v>
       </c>
       <c r="J23" s="2">
-        <v>46199.12570188512</v>
+        <v>46210.99822586024</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -1582,10 +1582,10 @@
         <v>1</v>
       </c>
       <c r="I24">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J24" s="2">
-        <v>46199.12571123514</v>
+        <v>46210.99823647695</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -1633,10 +1633,10 @@
         <v>1</v>
       </c>
       <c r="I25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J25" s="2">
-        <v>46199.12571191258</v>
+        <v>46210.99823752359</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -1780,10 +1780,10 @@
         <v>1</v>
       </c>
       <c r="I28">
-        <v>150.4</v>
+        <v>150.7</v>
       </c>
       <c r="J28" s="2">
-        <v>46210.58447072034</v>
+        <v>46210.63096642157</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>

</xml_diff>